<commit_message>
Updated calculations and formatting for COCOMO I & II Calculations for Sprints 1, 2, 3 and 4.
</commit_message>
<xml_diff>
--- a/Evidence/PP/COCOMO I and II Calculations/COCOMO I & II Calculations Sprint 1.xlsx
+++ b/Evidence/PP/COCOMO I and II Calculations/COCOMO I & II Calculations Sprint 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neelp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{390CF3F5-EBEE-47DB-8259-8655EC33C500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B544598-C516-455B-B779-D6CF40ABFB2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8C05499B-E777-4CB1-ACAA-0667EC699DC3}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{8C05499B-E777-4CB1-ACAA-0667EC699DC3}"/>
   </bookViews>
   <sheets>
     <sheet name="COCOMO I and II" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="78">
   <si>
     <t>COCOMO I</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>File name</t>
-  </si>
-  <si>
-    <t>__init__</t>
   </si>
   <si>
     <t>LOC</t>
@@ -325,6 +322,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0E351C2F-CAAF-432A-BEE2-983DCE9A4234}" name="Table1" displayName="Table1" ref="A22:F40" totalsRowShown="0">
+  <autoFilter ref="A22:F40" xr:uid="{0E351C2F-CAAF-432A-BEE2-983DCE9A4234}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{9BEF8EFE-4E29-4188-AA78-27F80C4F9F50}" name="File name"/>
+    <tableColumn id="2" xr3:uid="{5E5637E1-3272-4834-97B7-B8C07B390932}" name="LOC"/>
+    <tableColumn id="3" xr3:uid="{012BCB08-3351-41E4-AB24-9ECDFD06CCC4}" name="KLOC"/>
+    <tableColumn id="4" xr3:uid="{2060EF71-73F3-4092-AABF-30C855AF4113}" name="E (Without EAF)"/>
+    <tableColumn id="5" xr3:uid="{77EA4941-96F7-4A35-BAA6-83F5A9E60E3F}" name="D (Without EAF)"/>
+    <tableColumn id="6" xr3:uid="{5B161F3C-4EAB-4AF5-A709-563317FA72D0}" name="P (Without EAF"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -644,15 +656,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEAEC6C2-1035-40B4-B580-094FC01FC123}">
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.26953125" customWidth="1"/>
     <col min="2" max="2" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.54296875" customWidth="1"/>
-    <col min="4" max="4" width="13.90625" customWidth="1"/>
-    <col min="5" max="5" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.35">
@@ -662,7 +674,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H2" t="s">
         <v>6</v>
@@ -682,7 +694,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="H3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I3">
         <v>2.4</v>
@@ -699,183 +711,183 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" t="s">
         <v>38</v>
       </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5">
         <v>1.1499999999999999</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7">
         <v>1.1499999999999999</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B17">
         <v>0.95</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B18">
         <v>0.91</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19">
         <v>1.1000000000000001</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B20">
         <f>PRODUCT(B5:B19)</f>
@@ -887,29 +899,24 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22" t="s">
         <v>1</v>
       </c>
       <c r="D22" t="s">
+        <v>42</v>
+      </c>
+      <c r="E22" t="s">
         <v>43</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>44</v>
-      </c>
-      <c r="F22" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B24">
         <v>120</v>
@@ -933,7 +940,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B25">
         <v>5</v>
@@ -957,7 +964,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B26">
         <v>80</v>
@@ -981,7 +988,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27">
         <v>90</v>
@@ -1005,7 +1012,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B28">
         <v>60</v>
@@ -1029,7 +1036,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B29">
         <v>50</v>
@@ -1053,7 +1060,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B30">
         <v>80</v>
@@ -1077,7 +1084,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B31">
         <v>180</v>
@@ -1101,7 +1108,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B32">
         <v>40</v>
@@ -1125,7 +1132,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B33">
         <v>15</v>
@@ -1149,7 +1156,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B34">
         <v>20</v>
@@ -1173,7 +1180,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B35">
         <v>65</v>
@@ -1197,7 +1204,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B36">
         <v>30</v>
@@ -1221,12 +1228,12 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B39">
         <f>SUM(B24:B36)</f>
@@ -1251,7 +1258,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B40">
         <f>B39</f>
@@ -1274,31 +1281,53 @@
         <v>0.70555673539278252</v>
       </c>
     </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>53</v>
+      </c>
+    </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="B45" t="s">
+        <v>38</v>
+      </c>
+      <c r="C45" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>56</v>
+      </c>
+      <c r="B46">
+        <v>3.72</v>
+      </c>
+      <c r="C46" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>56</v>
-      </c>
-      <c r="B47" t="s">
-        <v>39</v>
+        <v>57</v>
+      </c>
+      <c r="B47">
+        <v>3.04</v>
       </c>
       <c r="C47" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B48">
-        <v>3.72</v>
+        <v>4.24</v>
       </c>
       <c r="C48" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1306,43 +1335,30 @@
         <v>58</v>
       </c>
       <c r="B49">
-        <v>3.04</v>
+        <v>2.19</v>
       </c>
       <c r="C49" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B50">
-        <v>4.24</v>
+        <v>6.24</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B51">
-        <v>2.19</v>
-      </c>
-      <c r="C51" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52">
-        <v>6.24</v>
-      </c>
-      <c r="C52" t="s">
-        <v>64</v>
+        <f>SUM(B46:B50)</f>
+        <v>19.43</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -1350,86 +1366,80 @@
         <v>66</v>
       </c>
       <c r="B53">
-        <f>SUM(B48:B52)</f>
+        <f>C39</f>
+        <v>0.83499999999999996</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54">
+        <f>B51</f>
         <v>19.43</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B55">
-        <f>C39</f>
-        <v>0.83499999999999996</v>
+        <f>B20</f>
+        <v>1.2576313750000001</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>68</v>
-      </c>
-      <c r="B56">
-        <f>B53</f>
-        <v>19.43</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
         <v>69</v>
       </c>
-      <c r="B57">
-        <f>B20</f>
-        <v>1.2576313750000001</v>
+      <c r="B56" t="s">
+        <v>71</v>
+      </c>
+      <c r="C56" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
+        <v>64</v>
+      </c>
+      <c r="B58">
+        <f>2.4*B55*(B53)^(1.05+(0.01*B54))</f>
+        <v>2.4116766949494486</v>
+      </c>
+      <c r="C58" t="s">
         <v>70</v>
       </c>
-      <c r="B58" t="s">
-        <v>72</v>
-      </c>
-      <c r="C58" t="s">
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>73</v>
+      </c>
+      <c r="B59">
+        <f>2.5*(B58)^0.38</f>
+        <v>3.4931823858681361</v>
+      </c>
+      <c r="C59" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B60">
-        <f>2.4*B57*(B55)^(1.05+(0.01*B56))</f>
-        <v>2.4116766949494486</v>
+        <f xml:space="preserve"> B58/B59</f>
+        <v>0.69039529819743195</v>
       </c>
       <c r="C60" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>74</v>
-      </c>
-      <c r="B61">
-        <f>2.5*(B60)^0.38</f>
-        <v>3.4931823858681361</v>
-      </c>
-      <c r="C61" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
         <v>76</v>
-      </c>
-      <c r="B62">
-        <f xml:space="preserve"> B60/B61</f>
-        <v>0.69039529819743195</v>
-      </c>
-      <c r="C62" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>